<commit_message>
GMAC 3dB Class B Ru39/Rv39: 10K CW high-confidence results
Near-capacity rate point shows slow waterfall:
N=1024 BLER=0.023 (231 errors, HIGH confidence)
All N>=128 now have 10K CW with 200+ errors each.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/gmac_snr3dB/gmac_snr3dB_classB_Ru39_Rv39_SC/classB_Ru39_Rv39_snr3dB_SC.xlsx
+++ b/results/gmac_snr3dB/gmac_snr3dB_classB_Ru39_Rv39_SC/classB_Ru39_Rv39_snr3dB_SC.xlsx
@@ -16,10 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
-  </numFmts>
-  <fonts count="5">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,40 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -68,30 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,283 +415,275 @@
   </sheetPr>
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Gaussian MAC — Class B, (Ru=0.39, Rv=0.39), SNR=3dB, SC (L=1)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Symmetric capacity: Rx=Ry ≤ 0.5548 bits/use | Sum capacity: 1.1095 bits/use | Path: 0^(N/2) 1^N 0^(N/2)</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>ku</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>kv</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Ru</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Rv</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Sum Rate</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>BLER</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Codewords</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" t="n">
         <v>0.375</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" t="n">
         <v>0.375</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" t="n">
         <v>0.75</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" t="n">
         <v>0.1496</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" t="n">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" t="n">
         <v>0.375</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" t="n">
         <v>0.375</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" t="n">
         <v>0.75</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" t="n">
         <v>0.1802</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" t="n">
         <v>12</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" t="n">
         <v>0.375</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" t="n">
         <v>0.375</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" t="n">
         <v>0.75</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" t="n">
         <v>0.2098</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" t="n">
         <v>64</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" t="n">
         <v>0.3906</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" t="n">
         <v>0.3906</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" t="n">
         <v>0.7812</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" t="n">
         <v>0.1532</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" t="n">
         <v>128</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" t="n">
         <v>50</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" t="n">
         <v>50</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" t="n">
         <v>0.3906</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" t="n">
         <v>0.3906</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" t="n">
         <v>0.7812</v>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>0.1368</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>5000</v>
+      <c r="G9" t="n">
+        <v>0.1398</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" t="n">
         <v>256</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" t="n">
         <v>99</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" t="n">
         <v>99</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" t="n">
         <v>0.3867</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" t="n">
         <v>0.3867</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" t="n">
         <v>0.7734</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>0.08840000000000001</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>5000</v>
+      <c r="G10" t="n">
+        <v>0.09130000000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" t="n">
         <v>512</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" t="n">
         <v>199</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" t="n">
         <v>199</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" t="n">
         <v>0.3887</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" t="n">
         <v>0.3887</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" t="n">
         <v>0.7773</v>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>0.0588</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>5000</v>
+      <c r="G11" t="n">
+        <v>0.0557</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" t="n">
         <v>1024</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" t="n">
         <v>398</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" t="n">
         <v>398</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" t="n">
         <v>0.3887</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" t="n">
         <v>0.3887</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" t="n">
         <v>0.7773</v>
       </c>
-      <c r="G12" s="5" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>3000</v>
-      </c>
-    </row>
+      <c r="G12" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="H12" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Capacity: I(Z;X)=0.3889, I(Z;Y|X)=0.7207, I(Z;X,Y)=1.1095</t>
         </is>

</xml_diff>